<commit_message>
Fase 4: correccion ortografica de catalogo, busqueda insensible a diacriticos y mejoras de exportacion y papelera
- Saneamiento de categoría CÀLCULO a CÁLCULO y actualización de claves foráneas
- Corrección de 36 rubros con tildes invertidas y errores ortográficos en item_catalog y seed-data
- Normalización preventiva en arranque con DatabaseSeedService.sanitizeCatalogAccents
- Búsqueda inteligente multi-palabra e insensible a diacríticos (tildes) en catálogo y clientes
- Formato monetario con prefijo '$' en atributos financieros de Excel y PDF
- Selector interactivo de columnas visibles con persistencia en localStorage en historial
- Borrado físico recursivo de carpetas en almacenamiento al eliminar definitivamente de papelera
- Calibración de paleta y opacidad ergonómica en botones de acción y papelera
</commit_message>
<xml_diff>
--- a/backend/seed-data/productos.xlsx
+++ b/backend/seed-data/productos.xlsx
@@ -1,34 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gt\Documents\Sexto Semestre-3 de Septimo - 06-04-2026\Sexto\Desarrollo De Sistemas de Informacion\construmetrica creacion de programa sobre la preformas\ContruProformas\backend\seed-data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F219250-E1D4-4303-8122-833794127EE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="14303" yWindow="-2490" windowWidth="19394" windowHeight="11475" xr2:uid="{3F7F2EB4-962A-4FE4-B40B-998D853C50D1}"/>
+    <workbookView xWindow="14303" yWindow="-2490" windowWidth="19394" windowHeight="11475"/>
   </bookViews>
   <sheets>
-    <sheet name="Productos1" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Productos1" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
@@ -80,13 +61,13 @@
     <t>A003</t>
   </si>
   <si>
-    <t>ALQUILER DE NIVEL AUTOMÀTICO</t>
+    <t>ALQUILER DE NIVEL AUTOMÁTICO</t>
   </si>
   <si>
     <t>A004</t>
   </si>
   <si>
-    <t>ALQUILER DE DRONE FOTOGRAMÈTRICO</t>
+    <t>ALQUILER DE DRONE FOTOGRAMÉTRICO</t>
   </si>
   <si>
     <t>A005</t>
@@ -101,7 +82,7 @@
     <t>COLOCACIONES</t>
   </si>
   <si>
-    <t>COLOCACIÒN DE PUNTOS DE CONTROL GEODESICO</t>
+    <t>COLOCACIÓN DE PUNTOS DE CONTROL GEODÉSICO</t>
   </si>
   <si>
     <t>C002</t>
@@ -131,7 +112,7 @@
     <t>C011</t>
   </si>
   <si>
-    <t>CREACION DE OBJETOS SIG</t>
+    <t>CREACIÓN DE OBJETOS SIG</t>
   </si>
   <si>
     <t>C013</t>
@@ -149,22 +130,22 @@
     <t>CA001</t>
   </si>
   <si>
-    <t>CÀLCULO</t>
-  </si>
-  <si>
-    <t>CÀLCULO ESTRUCTURAL POR M2</t>
+    <t>CÁLCULO</t>
+  </si>
+  <si>
+    <t>CÁLCULO ESTRUCTURAL POR M2</t>
   </si>
   <si>
     <t>CA002</t>
   </si>
   <si>
-    <t>MEDICION DE AREAS</t>
+    <t>MEDICIÓN DE ÁREAS</t>
   </si>
   <si>
     <t>CO010</t>
   </si>
   <si>
-    <t>CATASTRO DE SISTEMA DE DESAGUE</t>
+    <t>CATASTRO DE SISTEMA DE DESAGÜE</t>
   </si>
   <si>
     <t>CO11</t>
@@ -182,7 +163,7 @@
     <t>COO6</t>
   </si>
   <si>
-    <t>CALCULO DE VOLUMENES DE TIERRA</t>
+    <t>CÁLCULO DE VOLÚMENES DE TIERRA</t>
   </si>
   <si>
     <t>COO9</t>
@@ -197,7 +178,7 @@
     <t>DISEÑOS</t>
   </si>
   <si>
-    <t>DISEÑO HIDRAÙLICO SANITARIO</t>
+    <t>DISEÑO HIDRÁULICO SANITARIO</t>
   </si>
   <si>
     <t>D002</t>
@@ -251,19 +232,19 @@
     <t>E002</t>
   </si>
   <si>
-    <t>ELABORACIOÒN DE PLANOS ARCGIS</t>
+    <t>ELABORACIÓN DE PLANOS ARCGIS</t>
   </si>
   <si>
     <t>E003</t>
   </si>
   <si>
-    <t>ELABORACIÒN DE MONOGRAFÌAS DE PUNTOS DE CONTROL GEODÈSICO</t>
+    <t>ELABORACIÓN DE MONOGRAFÍAS DE PUNTOS DE CONTROL GEODÉSICO</t>
   </si>
   <si>
     <t>E004</t>
   </si>
   <si>
-    <t>CONSULTORIA DE ESTUDIOS</t>
+    <t>CONSULTORÍA DE ESTUDIOS</t>
   </si>
   <si>
     <t>E005</t>
@@ -281,19 +262,19 @@
     <t>E007</t>
   </si>
   <si>
-    <t>CONSULTORIA DE ESTUDIOS DE TOPOGRAFIA</t>
+    <t>CONSULTORÍA DE ESTUDIOS DE TOPOGRAFÍA</t>
   </si>
   <si>
     <t>E008</t>
   </si>
   <si>
-    <t>TOPOGRAFIA</t>
+    <t>TOPOGRAFÍA</t>
   </si>
   <si>
     <t>E009</t>
   </si>
   <si>
-    <t>PLANOS DE CONTEO DE ARBOLES</t>
+    <t>PLANOS DE CONTEO DE ÁRBOLES</t>
   </si>
   <si>
     <t>E010</t>
@@ -305,13 +286,13 @@
     <t>E011</t>
   </si>
   <si>
-    <t>ASBUILD DE ALCANTARILLADO Y AGUA POTABLE</t>
+    <t>AS-BUILT DE ALCANTARILLADO Y AGUA POTABLE</t>
   </si>
   <si>
     <t>E012</t>
   </si>
   <si>
-    <t>ASBUILD ÉLECTRICO</t>
+    <t>AS-BUILT ELÉCTRICO</t>
   </si>
   <si>
     <t>E013</t>
@@ -335,13 +316,13 @@
     <t>E016</t>
   </si>
   <si>
-    <t>ESTUDIO DE MECANICA DE SUELOS</t>
+    <t>ESTUDIO DE MECÁNICA DE SUELOS</t>
   </si>
   <si>
     <t>E017</t>
   </si>
   <si>
-    <t>GEOTÉCNIA</t>
+    <t>GEOTECNIA</t>
   </si>
   <si>
     <t>E018</t>
@@ -353,25 +334,25 @@
     <t>E019</t>
   </si>
   <si>
-    <t>INFORME GEOTECNIA</t>
+    <t>INFORME DE GEOTECNIA</t>
   </si>
   <si>
     <t>E020</t>
   </si>
   <si>
-    <t>CÁLCULO DE VOLUMENES</t>
+    <t>CÁLCULO DE VOLÚMENES</t>
   </si>
   <si>
     <t>E021</t>
   </si>
   <si>
-    <t>EVALUACIÓN DEL SISTEMA DE ALCANTARRILLADO</t>
+    <t>EVALUACIÓN DEL SISTEMA DE ALCANTARILLADO</t>
   </si>
   <si>
     <t>E022</t>
   </si>
   <si>
-    <t>ELABORACION DE ORTOFOTO</t>
+    <t>ELABORACIÓN DE ORTOFOTO</t>
   </si>
   <si>
     <t>E023</t>
@@ -419,7 +400,7 @@
     <t>E030</t>
   </si>
   <si>
-    <t>LÍNEA SISMICA</t>
+    <t>LÍNEA SÍSMICA</t>
   </si>
   <si>
     <t>E031</t>
@@ -437,7 +418,7 @@
     <t>E034</t>
   </si>
   <si>
-    <t>PESO ESPECIFÍCO DEL SUELO</t>
+    <t>PESO ESPECÍFICO DEL SUELO</t>
   </si>
   <si>
     <t>L001</t>
@@ -446,7 +427,7 @@
     <t>LEVANTAMIENTOS</t>
   </si>
   <si>
-    <t>LEVANTAMIENTO PLANIMÈTRICO X M2</t>
+    <t>LEVANTAMIENTO PLANIMÉTRICO X M2</t>
   </si>
   <si>
     <t>L002</t>
@@ -464,7 +445,7 @@
     <t>L004</t>
   </si>
   <si>
-    <t>LEVANTAMIENTO AEROFOTOGRAMÈTRICO CON DRONE</t>
+    <t>LEVANTAMIENTO AEROFOTOGRAMÉTRICO CON DRONE</t>
   </si>
   <si>
     <t>L005</t>
@@ -509,7 +490,7 @@
     <t>LEVANTAMIENTO LIDAR</t>
   </si>
   <si>
-    <t>l012</t>
+    <t>L012</t>
   </si>
   <si>
     <t>VUELO CON DRON</t>
@@ -545,7 +526,7 @@
     <t>RECORRIDOS</t>
   </si>
   <si>
-    <t>RECORRIDO DE LINDERO CON ESTACIÒN TOTAL</t>
+    <t>RECORRIDO DE LINDERO CON ESTACIÓN TOTAL</t>
   </si>
   <si>
     <t>R002</t>
@@ -557,7 +538,7 @@
     <t>R003</t>
   </si>
   <si>
-    <t>VIATICOS Y SUBSISTENCIAS</t>
+    <t>VIÁTICOS Y SUBSISTENCIAS</t>
   </si>
   <si>
     <t>RP001</t>
@@ -587,7 +568,7 @@
     <t>RP005</t>
   </si>
   <si>
-    <t>REPLANTEO TOPOGRAFICO(PLANIMETRIA)</t>
+    <t>REPLANTEO TOPOGRÁFICO (PLANIMETRÍA)</t>
   </si>
   <si>
     <t>RP006</t>
@@ -614,13 +595,13 @@
     <t>TRÁMITES</t>
   </si>
   <si>
-    <t>TRÀMITE DE REGULACIÒN DE ÀREAS</t>
+    <t>TRÁMITE DE REGULACIÓN DE ÁREAS</t>
   </si>
   <si>
     <t>T002</t>
   </si>
   <si>
-    <t>TRÀMITE DE UBICACIÒN GEOGRÀFICA DE LOTE</t>
+    <t>TRÁMITE DE UBICACIÓN GEOGRÁFICA DE LOTE</t>
   </si>
   <si>
     <t>T003</t>
@@ -638,7 +619,7 @@
     <t>T005</t>
   </si>
   <si>
-    <t>TRAMITE DE APROBACIÓN</t>
+    <t>TRÁMITE DE APROBACIÓN</t>
   </si>
   <si>
     <t>T006</t>
@@ -665,41 +646,37 @@
     <t>VISITAS</t>
   </si>
   <si>
-    <t>VISITA TÈCNICA Y RECONOCIMIENTO</t>
+    <t>VISITA TÉCNICA Y RECONOCIMIENTO</t>
   </si>
   <si>
     <t>V002</t>
   </si>
   <si>
-    <t>MOVILIZACION DE EQUIPOS</t>
+    <t>MOVILIZACIÓN DE EQUIPOS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <charset val="1"/>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <charset val="1"/>
       <sz val="10"/>
       <name val="Verdana"/>
-      <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <charset val="1"/>
       <sz val="10"/>
       <name val="Verdana"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Verdana"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -720,15 +697,15 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1062,12 +1039,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FDCC3AC-2D97-4636-82D8-A80B12B02C49}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:D102"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="3" width="80" customWidth="1"/>
@@ -1075,1415 +1052,1415 @@
     <col min="5" max="256" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="B5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
+      <c r="D5" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
+      <c r="D6" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
+      <c r="D7" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
+      <c r="C8" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
+      <c r="D9" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
+      <c r="D11" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
+      <c r="D12" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
+      <c r="D13" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D14" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="2" t="s">
+      <c r="D14" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="2" t="s">
+      <c r="D15" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D16" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="2" t="s">
+      <c r="D16" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D17" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="2" t="s">
+      <c r="D17" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D18" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="2" t="s">
+      <c r="D18" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D19" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="2" t="s">
+      <c r="D19" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D20" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="2" t="s">
+      <c r="D20" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="2" t="s">
+      <c r="D21" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D22" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="2" t="s">
+      <c r="D22" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D23" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="2" t="s">
+      <c r="D23" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="D24" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="2" t="s">
+      <c r="D24" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D25" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="2" t="s">
+      <c r="D25" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D26" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="2" t="s">
+      <c r="D26" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D27" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="2" t="s">
+      <c r="D27" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C28" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D28" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="2" t="s">
+      <c r="D28" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="C29" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="D29" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="2" t="s">
+      <c r="D29" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="D30" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="2" t="s">
+      <c r="D30" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C31" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D31" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="2" t="s">
+      <c r="D31" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="D32" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="2" t="s">
+      <c r="D32" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="C33" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="D33" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="2" t="s">
+      <c r="D33" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C34" s="2" t="s">
+      <c r="B34" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C34" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="D34" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="2" t="s">
+      <c r="D34" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B35" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C35" s="2" t="s">
+      <c r="B35" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C35" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="D35" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" s="2" t="s">
+      <c r="D35" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C36" s="2" t="s">
+      <c r="B36" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C36" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="D36" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" s="2" t="s">
+      <c r="D36" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C37" s="2" t="s">
+      <c r="B37" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C37" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="D37" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="2" t="s">
+      <c r="D37" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B38" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C38" s="2" t="s">
+      <c r="B38" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C38" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="D38" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="2" t="s">
+      <c r="D38" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B39" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C39" s="2" t="s">
+      <c r="B39" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C39" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="D39" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="2" t="s">
+      <c r="D39" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B40" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C40" s="2" t="s">
+      <c r="B40" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C40" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="D40" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="2" t="s">
+      <c r="D40" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="B41" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C41" s="2" t="s">
+      <c r="B41" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C41" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="D41" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="2" t="s">
+      <c r="D41" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B42" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C42" s="2" t="s">
+      <c r="B42" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="D42" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A43" s="2" t="s">
+      <c r="D42" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B43" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C43" s="2" t="s">
+      <c r="B43" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C43" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="D43" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A44" s="2" t="s">
+      <c r="D43" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B44" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C44" s="2" t="s">
+      <c r="B44" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C44" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="D44" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="2" t="s">
+      <c r="D44" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="B45" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C45" s="2" t="s">
+      <c r="B45" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C45" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D45" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="2" t="s">
+      <c r="D45" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B46" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C46" s="2" t="s">
+      <c r="B46" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C46" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="D46" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="2" t="s">
+      <c r="D46" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="B47" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C47" s="2" t="s">
+      <c r="B47" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C47" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="D47" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A48" s="2" t="s">
+      <c r="D47" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="B48" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C48" s="2" t="s">
+      <c r="B48" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C48" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D48" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" s="2" t="s">
+      <c r="D48" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="B49" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C49" s="2" t="s">
+      <c r="B49" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C49" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="D49" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A50" s="2" t="s">
+      <c r="D49" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="B50" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C50" s="2" t="s">
+      <c r="B50" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C50" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="D50" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A51" s="2" t="s">
+      <c r="D50" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="B51" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C51" s="2" t="s">
+      <c r="B51" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C51" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="D51" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" s="2" t="s">
+      <c r="D51" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="B52" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C52" s="2" t="s">
+      <c r="B52" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C52" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="D52" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" s="2" t="s">
+      <c r="D52" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="B53" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C53" s="2" t="s">
+      <c r="B53" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C53" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="D53" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" s="2" t="s">
+      <c r="D53" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="B54" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C54" s="2" t="s">
+      <c r="B54" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C54" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="D54" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A55" s="2" t="s">
+      <c r="D54" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="B55" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C55" s="2" t="s">
+      <c r="B55" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C55" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="D55" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A56" s="2" t="s">
+      <c r="D55" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="B56" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C56" s="2" t="s">
+      <c r="B56" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C56" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="D56" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A57" s="2" t="s">
+      <c r="D56" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="B57" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C57" s="2" t="s">
+      <c r="B57" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C57" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="D57" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A58" s="2" t="s">
+      <c r="D57" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="B58" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C58" s="2" t="s">
+      <c r="B58" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C58" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="D58" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A59" s="2" t="s">
+      <c r="D58" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="B59" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C59" s="2" t="s">
+      <c r="B59" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C59" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="D59" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" s="2" t="s">
+      <c r="D59" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="B60" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C60" s="2" t="s">
+      <c r="B60" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C60" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="D60" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A61" s="2" t="s">
+      <c r="D60" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="B61" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C61" s="2" t="s">
+      <c r="B61" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C61" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="D61" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" s="2" t="s">
+      <c r="D61" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B62" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C62" s="2" t="s">
+      <c r="B62" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C62" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="D62" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" s="2" t="s">
+      <c r="D62" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B63" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C63" s="2" t="s">
+      <c r="B63" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C63" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="D63" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" s="2" t="s">
+      <c r="D63" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="B64" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C64" s="2" t="s">
+      <c r="B64" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C64" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="D64" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A65" s="2" t="s">
+      <c r="D64" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="B65" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C65" s="2" t="s">
+      <c r="B65" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C65" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="D65" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A66" s="2" t="s">
+      <c r="D65" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="B66" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C66" s="2" t="s">
+      <c r="B66" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C66" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="D66" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A67" s="2" t="s">
+      <c r="D66" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="B67" s="2" t="s">
+      <c r="B67" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C67" s="2" t="s">
+      <c r="C67" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="D67" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" s="2" t="s">
+      <c r="D67" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="B68" s="2" t="s">
+      <c r="B68" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C68" s="2" t="s">
+      <c r="C68" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="D68" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A69" s="2" t="s">
+      <c r="D68" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="B69" s="2" t="s">
+      <c r="B69" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C69" s="2" t="s">
+      <c r="C69" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="D69" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" s="2" t="s">
+      <c r="D69" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="B70" s="2" t="s">
+      <c r="B70" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C70" s="2" t="s">
+      <c r="C70" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="D70" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A71" s="2" t="s">
+      <c r="D70" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="B71" s="2" t="s">
+      <c r="B71" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C71" s="2" t="s">
+      <c r="C71" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="D71" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A72" s="2" t="s">
+      <c r="D71" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="B72" s="2" t="s">
+      <c r="B72" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C72" s="2" t="s">
+      <c r="C72" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="D72" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A73" s="2" t="s">
+      <c r="D72" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="B73" s="2" t="s">
+      <c r="B73" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C73" s="2" t="s">
+      <c r="C73" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="D73" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" s="2" t="s">
+      <c r="D73" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="B74" s="2" t="s">
+      <c r="B74" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C74" s="2" t="s">
+      <c r="C74" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="D74" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A75" s="2" t="s">
+      <c r="D74" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="B75" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C75" s="2" t="s">
+      <c r="C75" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="D75" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A76" s="2" t="s">
+      <c r="D75" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="B76" s="2" t="s">
+      <c r="B76" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C76" s="2" t="s">
+      <c r="C76" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="D76" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" s="2" t="s">
+      <c r="D76" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="B77" s="2" t="s">
+      <c r="B77" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C77" s="2" t="s">
+      <c r="C77" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="D77" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A78" s="2" t="s">
+      <c r="D77" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="B78" s="2" t="s">
+      <c r="B78" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C78" s="2" t="s">
+      <c r="C78" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="D78" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A79" s="2" t="s">
+      <c r="D78" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="B79" s="2" t="s">
+      <c r="B79" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="C79" s="2" t="s">
+      <c r="C79" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="D79" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A80" s="2" t="s">
+      <c r="D79" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="B80" s="2" t="s">
+      <c r="B80" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="C80" s="2" t="s">
+      <c r="C80" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="D80" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A81" s="2" t="s">
+      <c r="D80" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="B81" s="2" t="s">
+      <c r="B81" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="C81" s="2" t="s">
+      <c r="C81" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="D81" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A82" s="2" t="s">
+      <c r="D81" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="B82" s="2" t="s">
+      <c r="B82" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="C82" s="2" t="s">
+      <c r="C82" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="D82" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A83" s="2" t="s">
+      <c r="D82" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="B83" s="2" t="s">
+      <c r="B83" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="C83" s="2" t="s">
+      <c r="C83" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="D83" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A84" s="2" t="s">
+      <c r="D83" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="B84" s="2" t="s">
+      <c r="B84" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="C84" s="2" t="s">
+      <c r="C84" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="D84" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A85" s="2" t="s">
+      <c r="D84" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="B85" s="2" t="s">
+      <c r="B85" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="C85" s="2" t="s">
+      <c r="C85" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="D85" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A86" s="2" t="s">
+      <c r="D85" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="B86" s="2" t="s">
+      <c r="B86" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="C86" s="2" t="s">
+      <c r="C86" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="D86" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A87" s="2" t="s">
+      <c r="D86" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="B87" s="2" t="s">
+      <c r="B87" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="C87" s="2" t="s">
+      <c r="C87" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="D87" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A88" s="2" t="s">
+      <c r="D87" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="B88" s="2" t="s">
+      <c r="B88" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="C88" s="2" t="s">
+      <c r="C88" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="D88" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A89" s="2" t="s">
+      <c r="D88" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="B89" s="2" t="s">
+      <c r="B89" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="C89" s="2" t="s">
+      <c r="C89" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="D89" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A90" s="2" t="s">
+      <c r="D89" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="B90" s="2" t="s">
+      <c r="B90" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="C90" s="2" t="s">
+      <c r="C90" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="D90" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A91" s="2" t="s">
+      <c r="D90" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="B91" s="2" t="s">
+      <c r="B91" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="C91" s="2" t="s">
+      <c r="C91" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="D91" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A92" s="2" t="s">
+      <c r="D91" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A92" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="B92" s="2" t="s">
+      <c r="B92" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="C92" s="2" t="s">
+      <c r="C92" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="D92" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A93" s="2" t="s">
+      <c r="D92" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A93" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="B93" s="2" t="s">
+      <c r="B93" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="C93" s="2" t="s">
+      <c r="C93" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="D93" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A94" s="2" t="s">
+      <c r="D93" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A94" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="B94" s="2" t="s">
+      <c r="B94" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="C94" s="2" t="s">
+      <c r="C94" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="D94" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A95" s="2" t="s">
+      <c r="D94" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A95" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="B95" s="2" t="s">
+      <c r="B95" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="C95" s="2" t="s">
+      <c r="C95" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="D95" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A96" s="2" t="s">
+      <c r="D95" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A96" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="B96" s="2" t="s">
+      <c r="B96" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="C96" s="2" t="s">
+      <c r="C96" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="D96" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A97" s="2" t="s">
+      <c r="D96" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="B97" s="2" t="s">
+      <c r="B97" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="C97" s="2" t="s">
+      <c r="C97" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="D97" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A98" s="2" t="s">
+      <c r="D97" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="B98" s="2" t="s">
+      <c r="B98" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="C98" s="2" t="s">
+      <c r="C98" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="D98" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A99" s="2" t="s">
+      <c r="D98" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A99" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="B99" s="2" t="s">
+      <c r="B99" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="C99" s="2" t="s">
+      <c r="C99" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="D99" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A100" s="2" t="s">
+      <c r="D99" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A100" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="B100" s="2" t="s">
+      <c r="B100" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="C100" s="2" t="s">
+      <c r="C100" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="D100" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A101" s="2" t="s">
+      <c r="D100" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A101" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="B101" s="2" t="s">
+      <c r="B101" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="C101" s="2" t="s">
+      <c r="C101" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="D101" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A102" s="2" t="s">
+      <c r="D101" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="B102" s="2" t="s">
+      <c r="B102" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="C102" s="2" t="s">
+      <c r="C102" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="D102" s="2">
+      <c r="D102" s="3">
         <v>15</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A1:C1"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.61" bottom="0.37" header="0.1" footer="0.1"/>
-  <pageSetup paperSize="9" pageOrder="overThenDown" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
-  <headerFooter alignWithMargins="0">
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" pageOrder="overThenDown" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <headerFooter>
     <oddHeader>&amp;P</oddHeader>
     <oddFooter>&amp;F</oddFooter>
   </headerFooter>

</xml_diff>